<commit_message>
docs(data): dong bo data_manifest.json + data_dictionary.xlsx voi CLI hien tai
data_manifest.json cu thieu entry price_limit_violations dau cli.py da ghi -
chay lai `qshield-data manifest --config configs/base.yaml` de dong bo. Cung
cap nhat data_dictionary.xlsx (da co dong exchange_periods trong report.py
tu truoc nhung file .xlsx tracked chua duoc regenerate).

Khong dong data/metadata/universe_asof_20260803.csv: file do chi duoc
regenerate qua `qshield-data fetch`, lenh nay tai du lieu that tu
yfinance/DNSE/vnstock qua mang - ngoai pham vi nhanh nay, va la quyet dinh
cua data owner.
</commit_message>
<xml_diff>
--- a/data/metadata/data_dictionary.xlsx
+++ b/data/metadata/data_dictionary.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -600,7 +600,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Lịch sử chuyển sàn</t>
+          <t>Lịch sử chuyển sàn (văn xuôi)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -612,25 +612,52 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>exchange_periods</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>list[dict]</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Lịch sử chuyển sàn dạng máy đọc được, dùng để resolve biên độ giá theo ngày (quality.price_limits). Mỗi phần tử {exchange, from?, until?}, biên đóng. Phải khớp exchange_current ở period hiện hành.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>[{'exchange': 'HNX', 'until': '2020-11-30'}, {'exchange': 'HOSE', 'from': '2020-12-01'}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>data_source</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Nguồn tải giá chính: yahoo | dnse</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>dnse</t>
         </is>

</xml_diff>